<commit_message>
Update H10 FX workbook
</commit_message>
<xml_diff>
--- a/downloads/FRB_H10_2026-10-05_to_2026-10-09.xlsx
+++ b/downloads/FRB_H10_2026-10-05_to_2026-10-09.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -53,10 +55,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -514,6 +517,27 @@
           <t>2026-10-05</t>
         </is>
       </c>
+      <c r="B6" s="3" t="n">
+        <v>0.6969</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>1.1211</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>1.3217</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.5598</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>1.4244</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>96.29000000000001</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>4.085</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -521,6 +545,27 @@
           <t>2026-10-06</t>
         </is>
       </c>
+      <c r="B7" s="3" t="n">
+        <v>0.6984</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>1.1262</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>1.3281</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.5626</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>1.4219</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>96.42</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>4.0825</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -528,6 +573,27 @@
           <t>2026-10-07</t>
         </is>
       </c>
+      <c r="B8" s="3" t="n">
+        <v>0.6962</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>1.1187</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>1.3213</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0.5597</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>1.4255</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>96.76000000000001</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>4.086</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -535,12 +601,54 @@
           <t>2026-10-08</t>
         </is>
       </c>
+      <c r="B9" s="3" t="n">
+        <v>0.6949</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>1.1192</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>1.3211</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0.5594</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>1.4246</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>96.78</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>4.089</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0.6979</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>1.1193</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>1.3229</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0.5611</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>1.4269</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>96.73</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>4.083</v>
       </c>
     </row>
     <row r="13">

</xml_diff>